<commit_message>
Oct 11, 2026, 4:00 PM
</commit_message>
<xml_diff>
--- a/Ekstraklasa 2026-2027.xlsx
+++ b/Ekstraklasa 2026-2027.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3D35629-E86E-4495-9CD0-347BC84A87DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB14C2E0-7A91-464C-BEC3-F5F165618004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2135F1F7-09EA-48F3-B6CC-5B3344B37E4D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="188">
   <si>
     <t>date</t>
   </si>
@@ -598,6 +598,12 @@
   <si>
     <t>Sat 10 October, 14:45</t>
   </si>
+  <si>
+    <t>Sat 10 October, 17:30</t>
+  </si>
+  <si>
+    <t>Sat 10 October, 20:15</t>
+  </si>
 </sst>
 </file>
 
@@ -1008,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2594D30A-B571-44E9-871B-38CB8D593531}">
-  <dimension ref="A1:CJ82"/>
+  <dimension ref="A1:CJ84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.85546875" customWidth="1"/>
@@ -1343,7 +1349,7 @@
         <v>42</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H82" si="0">100-G2</f>
+        <f t="shared" ref="H2:H84" si="0">100-G2</f>
         <v>58</v>
       </c>
       <c r="I2" s="3">
@@ -5592,7 +5598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:88" ht="25.5">
+    <row r="18" spans="1:88">
       <c r="A18">
         <v>17</v>
       </c>
@@ -6927,7 +6933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:88" ht="25.5">
+    <row r="23" spans="1:88">
       <c r="A23">
         <v>22</v>
       </c>
@@ -7194,7 +7200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:88" ht="25.5">
+    <row r="24" spans="1:88">
       <c r="A24">
         <v>23</v>
       </c>
@@ -7995,7 +8001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:88" ht="25.5">
+    <row r="27" spans="1:88">
       <c r="A27">
         <v>26</v>
       </c>
@@ -8529,7 +8535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:88" ht="25.5">
+    <row r="29" spans="1:88">
       <c r="A29">
         <v>28</v>
       </c>
@@ -8796,7 +8802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:88" ht="25.5">
+    <row r="30" spans="1:88">
       <c r="A30">
         <v>29</v>
       </c>
@@ -10929,7 +10935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:88" ht="25.5">
+    <row r="38" spans="1:88">
       <c r="B38" s="4" t="s">
         <v>142</v>
       </c>
@@ -11193,7 +11199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:88" ht="25.5">
+    <row r="39" spans="1:88">
       <c r="B39" s="4" t="s">
         <v>143</v>
       </c>
@@ -12249,7 +12255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:88" ht="25.5">
+    <row r="43" spans="1:88">
       <c r="B43" s="2" t="s">
         <v>147</v>
       </c>
@@ -12777,7 +12783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:88" ht="25.5">
+    <row r="45" spans="1:88">
       <c r="B45" s="2" t="s">
         <v>149</v>
       </c>
@@ -13305,7 +13311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:88" ht="25.5">
+    <row r="47" spans="1:88">
       <c r="B47" s="4" t="s">
         <v>151</v>
       </c>
@@ -13569,7 +13575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:88" ht="25.5">
+    <row r="48" spans="1:88">
       <c r="B48" s="4" t="s">
         <v>152</v>
       </c>
@@ -22806,6 +22812,534 @@
         <v>0</v>
       </c>
       <c r="CJ82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="2:88">
+      <c r="B83" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="C83" t="s">
+        <v>99</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E83">
+        <v>1</v>
+      </c>
+      <c r="F83">
+        <v>4</v>
+      </c>
+      <c r="G83">
+        <v>40</v>
+      </c>
+      <c r="H83">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="I83">
+        <v>0.77</v>
+      </c>
+      <c r="J83">
+        <v>2.04</v>
+      </c>
+      <c r="K83">
+        <v>7</v>
+      </c>
+      <c r="L83">
+        <v>16</v>
+      </c>
+      <c r="M83">
+        <v>4</v>
+      </c>
+      <c r="N83">
+        <v>5</v>
+      </c>
+      <c r="O83">
+        <v>2</v>
+      </c>
+      <c r="P83">
+        <v>4</v>
+      </c>
+      <c r="Q83">
+        <v>1</v>
+      </c>
+      <c r="R83">
+        <v>2</v>
+      </c>
+      <c r="S83">
+        <v>251</v>
+      </c>
+      <c r="T83">
+        <v>444</v>
+      </c>
+      <c r="U83">
+        <v>13</v>
+      </c>
+      <c r="V83">
+        <v>11</v>
+      </c>
+      <c r="W83">
+        <v>3</v>
+      </c>
+      <c r="X83">
+        <v>4</v>
+      </c>
+      <c r="Y83" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z83" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA83">
+        <v>3</v>
+      </c>
+      <c r="AB83">
+        <v>5</v>
+      </c>
+      <c r="AC83">
+        <v>0</v>
+      </c>
+      <c r="AD83">
+        <v>6</v>
+      </c>
+      <c r="AE83">
+        <v>0</v>
+      </c>
+      <c r="AF83">
+        <v>0</v>
+      </c>
+      <c r="AG83">
+        <v>5</v>
+      </c>
+      <c r="AH83">
+        <v>12</v>
+      </c>
+      <c r="AI83">
+        <v>2</v>
+      </c>
+      <c r="AJ83">
+        <v>4</v>
+      </c>
+      <c r="AK83">
+        <v>0.63</v>
+      </c>
+      <c r="AL83">
+        <v>1.79</v>
+      </c>
+      <c r="AM83">
+        <v>0.13</v>
+      </c>
+      <c r="AN83">
+        <v>0.25</v>
+      </c>
+      <c r="AO83">
+        <v>0.77</v>
+      </c>
+      <c r="AP83">
+        <v>2.04</v>
+      </c>
+      <c r="AQ83">
+        <v>0.41</v>
+      </c>
+      <c r="AR83">
+        <v>2.6</v>
+      </c>
+      <c r="AS83">
+        <v>341</v>
+      </c>
+      <c r="AT83">
+        <v>517</v>
+      </c>
+      <c r="AU83">
+        <v>114</v>
+      </c>
+      <c r="AV83">
+        <v>225</v>
+      </c>
+      <c r="AW83">
+        <v>137</v>
+      </c>
+      <c r="AX83">
+        <v>219</v>
+      </c>
+      <c r="AY83">
+        <v>15</v>
+      </c>
+      <c r="AZ83">
+        <v>23</v>
+      </c>
+      <c r="BA83">
+        <v>3</v>
+      </c>
+      <c r="BB83">
+        <v>4</v>
+      </c>
+      <c r="BC83">
+        <v>15</v>
+      </c>
+      <c r="BD83">
+        <v>22</v>
+      </c>
+      <c r="BE83">
+        <v>22</v>
+      </c>
+      <c r="BF83">
+        <v>27</v>
+      </c>
+      <c r="BG83">
+        <v>2</v>
+      </c>
+      <c r="BH83">
+        <v>3</v>
+      </c>
+      <c r="BI83" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ83" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK83">
+        <v>16</v>
+      </c>
+      <c r="BL83">
+        <v>8</v>
+      </c>
+      <c r="BM83">
+        <v>10</v>
+      </c>
+      <c r="BN83">
+        <v>9</v>
+      </c>
+      <c r="BO83">
+        <v>6</v>
+      </c>
+      <c r="BP83">
+        <v>1</v>
+      </c>
+      <c r="BQ83">
+        <v>19</v>
+      </c>
+      <c r="BR83">
+        <v>30</v>
+      </c>
+      <c r="BS83">
+        <v>1</v>
+      </c>
+      <c r="BT83">
+        <v>2</v>
+      </c>
+      <c r="BU83" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV83" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW83">
+        <v>41</v>
+      </c>
+      <c r="BX83">
+        <v>37</v>
+      </c>
+      <c r="BY83">
+        <v>31</v>
+      </c>
+      <c r="BZ83">
+        <v>24</v>
+      </c>
+      <c r="CA83">
+        <v>10</v>
+      </c>
+      <c r="CB83">
+        <v>13</v>
+      </c>
+      <c r="CC83">
+        <v>5</v>
+      </c>
+      <c r="CD83">
+        <v>4</v>
+      </c>
+      <c r="CE83" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF83" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG83">
+        <v>2</v>
+      </c>
+      <c r="CH83">
+        <v>4</v>
+      </c>
+      <c r="CI83">
+        <v>0</v>
+      </c>
+      <c r="CJ83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="2:88" ht="30">
+      <c r="B84" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84">
+        <v>3</v>
+      </c>
+      <c r="G84">
+        <v>57</v>
+      </c>
+      <c r="H84">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="I84">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="J84">
+        <v>2.12</v>
+      </c>
+      <c r="K84">
+        <v>11</v>
+      </c>
+      <c r="L84">
+        <v>15</v>
+      </c>
+      <c r="M84">
+        <v>3</v>
+      </c>
+      <c r="N84">
+        <v>9</v>
+      </c>
+      <c r="O84">
+        <v>1</v>
+      </c>
+      <c r="P84">
+        <v>4</v>
+      </c>
+      <c r="Q84">
+        <v>1</v>
+      </c>
+      <c r="R84">
+        <v>1</v>
+      </c>
+      <c r="S84">
+        <v>400</v>
+      </c>
+      <c r="T84">
+        <v>289</v>
+      </c>
+      <c r="U84">
+        <v>13</v>
+      </c>
+      <c r="V84">
+        <v>18</v>
+      </c>
+      <c r="W84">
+        <v>4</v>
+      </c>
+      <c r="X84">
+        <v>4</v>
+      </c>
+      <c r="Y84" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z84" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA84">
+        <v>5</v>
+      </c>
+      <c r="AB84">
+        <v>2</v>
+      </c>
+      <c r="AC84">
+        <v>3</v>
+      </c>
+      <c r="AD84">
+        <v>4</v>
+      </c>
+      <c r="AE84">
+        <v>0</v>
+      </c>
+      <c r="AF84">
+        <v>0</v>
+      </c>
+      <c r="AG84">
+        <v>6</v>
+      </c>
+      <c r="AH84">
+        <v>14</v>
+      </c>
+      <c r="AI84">
+        <v>5</v>
+      </c>
+      <c r="AJ84">
+        <v>1</v>
+      </c>
+      <c r="AK84">
+        <v>0.52</v>
+      </c>
+      <c r="AL84">
+        <v>1.73</v>
+      </c>
+      <c r="AM84">
+        <v>0.05</v>
+      </c>
+      <c r="AN84">
+        <v>0.39</v>
+      </c>
+      <c r="AO84">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="AP84">
+        <v>2.12</v>
+      </c>
+      <c r="AQ84">
+        <v>0.96</v>
+      </c>
+      <c r="AR84">
+        <v>3.12</v>
+      </c>
+      <c r="AS84">
+        <v>496</v>
+      </c>
+      <c r="AT84">
+        <v>371</v>
+      </c>
+      <c r="AU84">
+        <v>234</v>
+      </c>
+      <c r="AV84">
+        <v>138</v>
+      </c>
+      <c r="AW84">
+        <v>166</v>
+      </c>
+      <c r="AX84">
+        <v>151</v>
+      </c>
+      <c r="AY84">
+        <v>30</v>
+      </c>
+      <c r="AZ84">
+        <v>27</v>
+      </c>
+      <c r="BA84">
+        <v>2</v>
+      </c>
+      <c r="BB84">
+        <v>4</v>
+      </c>
+      <c r="BC84">
+        <v>22</v>
+      </c>
+      <c r="BD84">
+        <v>15</v>
+      </c>
+      <c r="BE84">
+        <v>20</v>
+      </c>
+      <c r="BF84">
+        <v>30</v>
+      </c>
+      <c r="BG84">
+        <v>2</v>
+      </c>
+      <c r="BH84">
+        <v>0</v>
+      </c>
+      <c r="BI84" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ84" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK84">
+        <v>19</v>
+      </c>
+      <c r="BL84">
+        <v>11</v>
+      </c>
+      <c r="BM84">
+        <v>9</v>
+      </c>
+      <c r="BN84">
+        <v>10</v>
+      </c>
+      <c r="BO84">
+        <v>3</v>
+      </c>
+      <c r="BP84">
+        <v>3</v>
+      </c>
+      <c r="BQ84">
+        <v>27</v>
+      </c>
+      <c r="BR84">
+        <v>22</v>
+      </c>
+      <c r="BS84">
+        <v>6</v>
+      </c>
+      <c r="BT84">
+        <v>3</v>
+      </c>
+      <c r="BU84" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV84" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW84">
+        <v>57</v>
+      </c>
+      <c r="BX84">
+        <v>48</v>
+      </c>
+      <c r="BY84">
+        <v>42</v>
+      </c>
+      <c r="BZ84">
+        <v>34</v>
+      </c>
+      <c r="CA84">
+        <v>15</v>
+      </c>
+      <c r="CB84">
+        <v>14</v>
+      </c>
+      <c r="CC84">
+        <v>5</v>
+      </c>
+      <c r="CD84">
+        <v>10</v>
+      </c>
+      <c r="CE84" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF84" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG84">
+        <v>2</v>
+      </c>
+      <c r="CH84">
+        <v>4</v>
+      </c>
+      <c r="CI84">
+        <v>0</v>
+      </c>
+      <c r="CJ84">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Oct 17, 2026, 11:33 AM
</commit_message>
<xml_diff>
--- a/Ekstraklasa 2026-2027.xlsx
+++ b/Ekstraklasa 2026-2027.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{13C4D69C-E7CE-4BCB-B506-7354E671E271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE96D956-CE20-403E-A9DD-353EA4F0C384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2135F1F7-09EA-48F3-B6CC-5B3344B37E4D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="195">
   <si>
     <t>date</t>
   </si>
@@ -619,6 +619,12 @@
   <si>
     <t>Mon 12 October, 20:30</t>
   </si>
+  <si>
+    <t>Fri 16 October, 18:00</t>
+  </si>
+  <si>
+    <t>Fri 16 October, 20:30</t>
+  </si>
 </sst>
 </file>
 
@@ -1029,7 +1035,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2594D30A-B571-44E9-871B-38CB8D593531}">
-  <dimension ref="A1:CJ89"/>
+  <dimension ref="A1:CJ91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.85546875" customWidth="1"/>
@@ -1364,7 +1370,7 @@
         <v>42</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H89" si="0">100-G2</f>
+        <f t="shared" ref="H2:H91" si="0">100-G2</f>
         <v>58</v>
       </c>
       <c r="I2" s="3">
@@ -24675,6 +24681,534 @@
         <v>0</v>
       </c>
       <c r="CJ89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="2:88" ht="30">
+      <c r="B90" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E90">
+        <v>1</v>
+      </c>
+      <c r="F90">
+        <v>2</v>
+      </c>
+      <c r="G90">
+        <v>53</v>
+      </c>
+      <c r="H90">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+      <c r="I90">
+        <v>1.53</v>
+      </c>
+      <c r="J90">
+        <v>2.66</v>
+      </c>
+      <c r="K90">
+        <v>14</v>
+      </c>
+      <c r="L90">
+        <v>23</v>
+      </c>
+      <c r="M90">
+        <v>3</v>
+      </c>
+      <c r="N90">
+        <v>13</v>
+      </c>
+      <c r="O90">
+        <v>3</v>
+      </c>
+      <c r="P90">
+        <v>4</v>
+      </c>
+      <c r="Q90">
+        <v>2</v>
+      </c>
+      <c r="R90">
+        <v>2</v>
+      </c>
+      <c r="S90">
+        <v>457</v>
+      </c>
+      <c r="T90">
+        <v>402</v>
+      </c>
+      <c r="U90">
+        <v>9</v>
+      </c>
+      <c r="V90">
+        <v>10</v>
+      </c>
+      <c r="W90">
+        <v>5</v>
+      </c>
+      <c r="X90">
+        <v>4</v>
+      </c>
+      <c r="Y90" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z90" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA90">
+        <v>8</v>
+      </c>
+      <c r="AB90">
+        <v>7</v>
+      </c>
+      <c r="AC90">
+        <v>3</v>
+      </c>
+      <c r="AD90">
+        <v>3</v>
+      </c>
+      <c r="AE90">
+        <v>1</v>
+      </c>
+      <c r="AF90">
+        <v>0</v>
+      </c>
+      <c r="AG90">
+        <v>9</v>
+      </c>
+      <c r="AH90">
+        <v>13</v>
+      </c>
+      <c r="AI90">
+        <v>5</v>
+      </c>
+      <c r="AJ90">
+        <v>10</v>
+      </c>
+      <c r="AK90">
+        <v>1.27</v>
+      </c>
+      <c r="AL90">
+        <v>1.73</v>
+      </c>
+      <c r="AM90">
+        <v>0.26</v>
+      </c>
+      <c r="AN90">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="AO90">
+        <v>1.53</v>
+      </c>
+      <c r="AP90">
+        <v>1.87</v>
+      </c>
+      <c r="AQ90">
+        <v>0.8</v>
+      </c>
+      <c r="AR90">
+        <v>2.8</v>
+      </c>
+      <c r="AS90">
+        <v>530</v>
+      </c>
+      <c r="AT90">
+        <v>481</v>
+      </c>
+      <c r="AU90">
+        <v>205</v>
+      </c>
+      <c r="AV90">
+        <v>206</v>
+      </c>
+      <c r="AW90">
+        <v>252</v>
+      </c>
+      <c r="AX90">
+        <v>196</v>
+      </c>
+      <c r="AY90">
+        <v>25</v>
+      </c>
+      <c r="AZ90">
+        <v>25</v>
+      </c>
+      <c r="BA90">
+        <v>8</v>
+      </c>
+      <c r="BB90">
+        <v>7</v>
+      </c>
+      <c r="BC90">
+        <v>13</v>
+      </c>
+      <c r="BD90">
+        <v>15</v>
+      </c>
+      <c r="BE90">
+        <v>33</v>
+      </c>
+      <c r="BF90">
+        <v>26</v>
+      </c>
+      <c r="BG90">
+        <v>0</v>
+      </c>
+      <c r="BH90">
+        <v>2</v>
+      </c>
+      <c r="BI90" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ90" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK90">
+        <v>9</v>
+      </c>
+      <c r="BL90">
+        <v>7</v>
+      </c>
+      <c r="BM90">
+        <v>11</v>
+      </c>
+      <c r="BN90">
+        <v>4</v>
+      </c>
+      <c r="BO90">
+        <v>2</v>
+      </c>
+      <c r="BP90">
+        <v>2</v>
+      </c>
+      <c r="BQ90">
+        <v>27</v>
+      </c>
+      <c r="BR90">
+        <v>23</v>
+      </c>
+      <c r="BS90">
+        <v>11</v>
+      </c>
+      <c r="BT90">
+        <v>2</v>
+      </c>
+      <c r="BU90" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV90" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW90">
+        <v>44</v>
+      </c>
+      <c r="BX90">
+        <v>43</v>
+      </c>
+      <c r="BY90">
+        <v>30</v>
+      </c>
+      <c r="BZ90">
+        <v>27</v>
+      </c>
+      <c r="CA90">
+        <v>14</v>
+      </c>
+      <c r="CB90">
+        <v>16</v>
+      </c>
+      <c r="CC90">
+        <v>11</v>
+      </c>
+      <c r="CD90">
+        <v>13</v>
+      </c>
+      <c r="CE90" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF90" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG90">
+        <v>3</v>
+      </c>
+      <c r="CH90">
+        <v>2</v>
+      </c>
+      <c r="CI90">
+        <v>0</v>
+      </c>
+      <c r="CJ90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="2:88">
+      <c r="B91" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E91">
+        <v>0</v>
+      </c>
+      <c r="F91">
+        <v>0</v>
+      </c>
+      <c r="G91">
+        <v>46</v>
+      </c>
+      <c r="H91">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="I91">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="J91">
+        <v>2.4900000000000002</v>
+      </c>
+      <c r="K91">
+        <v>10</v>
+      </c>
+      <c r="L91">
+        <v>21</v>
+      </c>
+      <c r="M91">
+        <v>3</v>
+      </c>
+      <c r="N91">
+        <v>4</v>
+      </c>
+      <c r="O91">
+        <v>0</v>
+      </c>
+      <c r="P91">
+        <v>3</v>
+      </c>
+      <c r="Q91">
+        <v>0</v>
+      </c>
+      <c r="R91">
+        <v>3</v>
+      </c>
+      <c r="S91">
+        <v>257</v>
+      </c>
+      <c r="T91">
+        <v>309</v>
+      </c>
+      <c r="U91">
+        <v>20</v>
+      </c>
+      <c r="V91">
+        <v>7</v>
+      </c>
+      <c r="W91">
+        <v>4</v>
+      </c>
+      <c r="X91">
+        <v>7</v>
+      </c>
+      <c r="Y91" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z91" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA91">
+        <v>3</v>
+      </c>
+      <c r="AB91">
+        <v>11</v>
+      </c>
+      <c r="AC91">
+        <v>4</v>
+      </c>
+      <c r="AD91">
+        <v>6</v>
+      </c>
+      <c r="AE91">
+        <v>1</v>
+      </c>
+      <c r="AF91">
+        <v>1</v>
+      </c>
+      <c r="AG91">
+        <v>3</v>
+      </c>
+      <c r="AH91">
+        <v>11</v>
+      </c>
+      <c r="AI91">
+        <v>7</v>
+      </c>
+      <c r="AJ91">
+        <v>10</v>
+      </c>
+      <c r="AK91">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="AL91">
+        <v>1.45</v>
+      </c>
+      <c r="AM91">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="AN91">
+        <v>0.25</v>
+      </c>
+      <c r="AO91">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="AP91">
+        <v>1.7</v>
+      </c>
+      <c r="AQ91">
+        <v>0.51</v>
+      </c>
+      <c r="AR91">
+        <v>0.32</v>
+      </c>
+      <c r="AS91">
+        <v>334</v>
+      </c>
+      <c r="AT91">
+        <v>400</v>
+      </c>
+      <c r="AU91">
+        <v>152</v>
+      </c>
+      <c r="AV91">
+        <v>151</v>
+      </c>
+      <c r="AW91">
+        <v>105</v>
+      </c>
+      <c r="AX91">
+        <v>158</v>
+      </c>
+      <c r="AY91">
+        <v>22</v>
+      </c>
+      <c r="AZ91">
+        <v>15</v>
+      </c>
+      <c r="BA91">
+        <v>2</v>
+      </c>
+      <c r="BB91">
+        <v>2</v>
+      </c>
+      <c r="BC91">
+        <v>23</v>
+      </c>
+      <c r="BD91">
+        <v>24</v>
+      </c>
+      <c r="BE91">
+        <v>16</v>
+      </c>
+      <c r="BF91">
+        <v>22</v>
+      </c>
+      <c r="BG91">
+        <v>2</v>
+      </c>
+      <c r="BH91">
+        <v>4</v>
+      </c>
+      <c r="BI91" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ91" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK91">
+        <v>20</v>
+      </c>
+      <c r="BL91">
+        <v>23</v>
+      </c>
+      <c r="BM91">
+        <v>19</v>
+      </c>
+      <c r="BN91">
+        <v>4</v>
+      </c>
+      <c r="BO91">
+        <v>5</v>
+      </c>
+      <c r="BP91">
+        <v>4</v>
+      </c>
+      <c r="BQ91">
+        <v>29</v>
+      </c>
+      <c r="BR91">
+        <v>12</v>
+      </c>
+      <c r="BS91">
+        <v>4</v>
+      </c>
+      <c r="BT91">
+        <v>3</v>
+      </c>
+      <c r="BU91" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV91" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW91">
+        <v>47</v>
+      </c>
+      <c r="BX91">
+        <v>55</v>
+      </c>
+      <c r="BY91">
+        <v>32</v>
+      </c>
+      <c r="BZ91">
+        <v>46</v>
+      </c>
+      <c r="CA91">
+        <v>15</v>
+      </c>
+      <c r="CB91">
+        <v>9</v>
+      </c>
+      <c r="CC91">
+        <v>5</v>
+      </c>
+      <c r="CD91">
+        <v>6</v>
+      </c>
+      <c r="CE91" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF91" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG91">
+        <v>4</v>
+      </c>
+      <c r="CH91">
+        <v>0</v>
+      </c>
+      <c r="CI91">
+        <v>0</v>
+      </c>
+      <c r="CJ91">
         <v>0</v>
       </c>
     </row>

</xml_diff>